<commit_message>
Session 14 handoff — thread_handoff.md merge + weekly_update duplicate guard + April 30 pipeline data
- thread_handoff.md: full merge of Sessions 11-14 (PT module, Backtest C, Sanchez fix, launch angle)
- weekly_update.py: _check_duplicate() guard prevents double-writing week column when pipeline hasn't refreshed
- data files: April 30 pipeline run (luck_scores, projections, pitcher scores, signal boards)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/signal_board_2026-04-29.xlsx
+++ b/outputs/signal_board_2026-04-29.xlsx
@@ -1751,12 +1751,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>92.8%</t>
+          <t>93.0%</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>92.8% rostered</t>
+          <t>93.0% rostered</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>92.3%</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>92.5% rostered</t>
+          <t>92.3% rostered</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1978,12 +1978,12 @@
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>91.0%</t>
+          <t>90.9%</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>91.0% rostered</t>
+          <t>90.9% rostered</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>88.8%</t>
+          <t>89.1%</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>88.8% rostered</t>
+          <t>89.1% rostered</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -2130,12 +2130,12 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>87.8% rostered</t>
+          <t>87.5% rostered</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -2207,12 +2207,12 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>86.0%</t>
+          <t>85.6%</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>86.0% rostered</t>
+          <t>85.6% rostered</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -2284,12 +2284,12 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>85.3%</t>
+          <t>85.5%</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>85.3% rostered</t>
+          <t>85.5% rostered</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -2361,12 +2361,12 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>83.1%</t>
+          <t>82.8%</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>83.1% rostered</t>
+          <t>82.8% rostered</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
@@ -2438,12 +2438,12 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>81.9%</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>82.5% rostered</t>
+          <t>81.9% rostered</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -2515,12 +2515,12 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>75.9%</t>
+          <t>74.7%</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>75.9% rostered</t>
+          <t>74.7% rostered</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
@@ -2592,12 +2592,12 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>70.9%</t>
+          <t>71.3%</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>70.9% rostered</t>
+          <t>71.3% rostered</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
@@ -2654,12 +2654,12 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Chase Delauter</t>
+          <t>Salvador Pérez</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -2669,12 +2669,12 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>69.8%</t>
+          <t>69.6%</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>69.8% rostered</t>
+          <t>69.6% rostered</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
@@ -2684,42 +2684,42 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>.327</t>
+          <t>.250</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>.376</t>
+          <t>.324</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>+.049</t>
+          <t>+.074</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>.228</t>
+          <t>.205</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.304</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-.099</t>
         </is>
       </c>
       <c r="M29" s="10" t="inlineStr">
         <is>
-          <t>+0.401</t>
+          <t>+0.176</t>
         </is>
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>36</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
@@ -2731,12 +2731,12 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Salvador Pérez</t>
+          <t>Chase Delauter</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -2746,12 +2746,12 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>69.5%</t>
+          <t>69.6%</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>69.5% rostered</t>
+          <t>69.6% rostered</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -2761,42 +2761,42 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>.327</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>.324</t>
+          <t>.376</t>
         </is>
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>+.074</t>
+          <t>+.049</t>
         </is>
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>.205</t>
+          <t>.228</t>
         </is>
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>.304</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L30" s="15" t="inlineStr">
         <is>
-          <t>-.099</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M30" s="14" t="inlineStr">
         <is>
-          <t>+0.176</t>
+          <t>+0.401</t>
         </is>
       </c>
       <c r="N30" s="13" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>25</t>
         </is>
       </c>
       <c r="O30" s="13" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>67.9%</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>68.5% rostered</t>
+          <t>67.9% rostered</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
@@ -2900,12 +2900,12 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>64.6%</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>63.0% rostered</t>
+          <t>64.6% rostered</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
@@ -2977,12 +2977,12 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>60.3%</t>
+          <t>60.1%</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>60.3% rostered</t>
+          <t>60.1% rostered</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -3054,12 +3054,12 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>51.0%</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>50.0% rostered</t>
+          <t>51.0% rostered</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
@@ -3131,12 +3131,12 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>45.0% rostered</t>
+          <t>44.4% rostered</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>42.8%</t>
+          <t>42.6%</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>42.8% rostered</t>
+          <t>42.6% rostered</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
@@ -3362,12 +3362,12 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>41.8%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>41.8% rostered</t>
+          <t>41.7% rostered</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
@@ -3439,12 +3439,12 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>36.8%</t>
+          <t>36.6%</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>36.8% rostered</t>
+          <t>36.6% rostered</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
@@ -3593,12 +3593,12 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>32.8%</t>
+          <t>32.7%</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>32.8% rostered</t>
+          <t>32.7% rostered</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -3670,12 +3670,12 @@
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>27.3%</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>26.9% rostered</t>
+          <t>27.3% rostered</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
@@ -3747,12 +3747,12 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>25.0% rostered</t>
+          <t>26.7% rostered</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
@@ -3824,12 +3824,12 @@
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>20.4% rostered</t>
+          <t>20.2% rostered</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
@@ -3901,12 +3901,12 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>17.2% rostered</t>
+          <t>17.1% rostered</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
@@ -3978,12 +3978,12 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>14.4% rostered</t>
+          <t>14.3% rostered</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
@@ -4055,12 +4055,12 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>13.7% rostered</t>
+          <t>13.6% rostered</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>13.1% rostered</t>
+          <t>13.0% rostered</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
@@ -4209,12 +4209,12 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>10.4% rostered</t>
+          <t>10.3% rostered</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>6.6% rostered</t>
+          <t>6.5% rostered</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
@@ -4425,12 +4425,12 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>Marcell Ozuna</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -4440,12 +4440,12 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>6.3% rostered</t>
+          <t>6.4% rostered</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
@@ -4455,42 +4455,42 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>.234</t>
+          <t>.319</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>.309</t>
+          <t>.369</t>
         </is>
       </c>
       <c r="I52" s="14" t="inlineStr">
         <is>
-          <t>+.075</t>
+          <t>+.050</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>.213</t>
+          <t>.250</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>.311</t>
+          <t>.293</t>
         </is>
       </c>
       <c r="L52" s="15" t="inlineStr">
         <is>
-          <t>-.099</t>
+          <t>-.043</t>
         </is>
       </c>
       <c r="M52" s="14" t="inlineStr">
         <is>
-          <t>+0.350</t>
+          <t>+0.242</t>
         </is>
       </c>
       <c r="N52" s="13" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>29</t>
         </is>
       </c>
       <c r="O52" s="13" t="inlineStr">
@@ -4502,12 +4502,12 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Marcell Ozuna</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -4532,42 +4532,42 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>.319</t>
+          <t>.234</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>.369</t>
+          <t>.309</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>+.050</t>
+          <t>+.075</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>.213</t>
         </is>
       </c>
       <c r="K53" s="8" t="inlineStr">
         <is>
-          <t>.293</t>
+          <t>.311</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
         <is>
-          <t>-.043</t>
+          <t>-.099</t>
         </is>
       </c>
       <c r="M53" s="10" t="inlineStr">
         <is>
-          <t>+0.242</t>
+          <t>+0.350</t>
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>36</t>
         </is>
       </c>
       <c r="O53" s="8" t="inlineStr">
@@ -4594,12 +4594,12 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>6.0% rostered</t>
+          <t>6.1% rostered</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
@@ -4748,12 +4748,12 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>5.1% rostered</t>
+          <t>5.0% rostered</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
@@ -4825,12 +4825,12 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.9%</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>5.0% rostered</t>
+          <t>4.9% rostered</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
@@ -5672,12 +5672,12 @@
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>82.2%</t>
+          <t>81.7%</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>82.2% rostered</t>
+          <t>81.7% rostered</t>
         </is>
       </c>
       <c r="F68" s="16" t="inlineStr">
@@ -5749,12 +5749,12 @@
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>34.7%</t>
+          <t>33.7%</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>34.7% rostered</t>
+          <t>33.7% rostered</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
@@ -5826,12 +5826,12 @@
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
         <is>
-          <t>16.6% rostered</t>
+          <t>16.4% rostered</t>
         </is>
       </c>
       <c r="F70" s="16" t="inlineStr">
@@ -5903,12 +5903,12 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>2.7%</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>2.8% rostered</t>
+          <t>2.7% rostered</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
@@ -6671,12 +6671,12 @@
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>97.2%</t>
+          <t>97.3%</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>97.2% rostered</t>
+          <t>97.3% rostered</t>
         </is>
       </c>
       <c r="F81" s="17" t="inlineStr">
@@ -6825,12 +6825,12 @@
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>94.4%</t>
+          <t>94.5%</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>94.4% rostered</t>
+          <t>94.5% rostered</t>
         </is>
       </c>
       <c r="F83" s="17" t="inlineStr">
@@ -6979,12 +6979,12 @@
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>85.9%</t>
+          <t>86.0%</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>85.9% rostered</t>
+          <t>86.0% rostered</t>
         </is>
       </c>
       <c r="F85" s="17" t="inlineStr">
@@ -7054,12 +7054,12 @@
       </c>
       <c r="D86" s="13" t="inlineStr">
         <is>
-          <t>84.2%</t>
+          <t>84.1%</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
         <is>
-          <t>84.2% rostered</t>
+          <t>84.1% rostered</t>
         </is>
       </c>
       <c r="F86" s="17" t="inlineStr">
@@ -7131,12 +7131,12 @@
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.9%</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>78.5% rostered</t>
+          <t>78.9% rostered</t>
         </is>
       </c>
       <c r="F87" s="17" t="inlineStr">
@@ -7208,12 +7208,12 @@
       </c>
       <c r="D88" s="13" t="inlineStr">
         <is>
-          <t>68.1%</t>
+          <t>67.8%</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
         <is>
-          <t>68.1% rostered</t>
+          <t>67.8% rostered</t>
         </is>
       </c>
       <c r="F88" s="17" t="inlineStr">
@@ -7285,12 +7285,12 @@
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>54.4%</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>54.5% rostered</t>
+          <t>54.4% rostered</t>
         </is>
       </c>
       <c r="F89" s="17" t="inlineStr">
@@ -7439,12 +7439,12 @@
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>38.4%</t>
+          <t>38.8%</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>38.4% rostered</t>
+          <t>38.8% rostered</t>
         </is>
       </c>
       <c r="F91" s="17" t="inlineStr">
@@ -7516,12 +7516,12 @@
       </c>
       <c r="D92" s="13" t="inlineStr">
         <is>
-          <t>30.5%</t>
+          <t>29.8%</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr">
         <is>
-          <t>30.5% rostered</t>
+          <t>29.8% rostered</t>
         </is>
       </c>
       <c r="F92" s="17" t="inlineStr">
@@ -7593,12 +7593,12 @@
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>28.0% rostered</t>
+          <t>29.4% rostered</t>
         </is>
       </c>
       <c r="F93" s="17" t="inlineStr">
@@ -7670,12 +7670,12 @@
       </c>
       <c r="D94" s="13" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr">
         <is>
-          <t>26.6% rostered</t>
+          <t>26.5% rostered</t>
         </is>
       </c>
       <c r="F94" s="17" t="inlineStr">
@@ -7747,12 +7747,12 @@
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>25.7% rostered</t>
+          <t>25.8% rostered</t>
         </is>
       </c>
       <c r="F95" s="17" t="inlineStr">
@@ -7824,12 +7824,12 @@
       </c>
       <c r="D96" s="13" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr">
         <is>
-          <t>20.7% rostered</t>
+          <t>22.8% rostered</t>
         </is>
       </c>
       <c r="F96" s="17" t="inlineStr">
@@ -7901,12 +7901,12 @@
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>9.0% rostered</t>
+          <t>8.3% rostered</t>
         </is>
       </c>
       <c r="F97" s="17" t="inlineStr">
@@ -7963,12 +7963,12 @@
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>Joey Wiemer</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -7978,12 +7978,12 @@
       </c>
       <c r="D98" s="13" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
         <is>
-          <t>8.3% rostered</t>
+          <t>8.1% rostered</t>
         </is>
       </c>
       <c r="F98" s="17" t="inlineStr">
@@ -7993,42 +7993,42 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>.374</t>
+          <t>.328</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>.303</t>
+          <t>.311</t>
         </is>
       </c>
       <c r="I98" s="15" t="inlineStr">
         <is>
-          <t>-.071</t>
+          <t>-.017</t>
         </is>
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>.458</t>
+          <t>.338</t>
         </is>
       </c>
       <c r="K98" s="13" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L98" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>.302</t>
+        </is>
+      </c>
+      <c r="L98" s="14" t="inlineStr">
+        <is>
+          <t>+.036</t>
         </is>
       </c>
       <c r="M98" s="15" t="inlineStr">
         <is>
-          <t>-0.111</t>
+          <t>-0.109</t>
         </is>
       </c>
       <c r="N98" s="13" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>24</t>
         </is>
       </c>
       <c r="O98" s="13" t="inlineStr">
@@ -8040,12 +8040,12 @@
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Joey Wiemer</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
@@ -8070,42 +8070,42 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>.328</t>
+          <t>.374</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>.311</t>
+          <t>.303</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>-.017</t>
+          <t>-.071</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>.338</t>
+          <t>.458</t>
         </is>
       </c>
       <c r="K99" s="8" t="inlineStr">
         <is>
-          <t>.302</t>
-        </is>
-      </c>
-      <c r="L99" s="10" t="inlineStr">
-        <is>
-          <t>+.036</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L99" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>-0.109</t>
+          <t>-0.111</t>
         </is>
       </c>
       <c r="N99" s="8" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="O99" s="8" t="inlineStr">
@@ -8132,12 +8132,12 @@
       </c>
       <c r="D100" s="13" t="inlineStr">
         <is>
-          <t>5.2%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="E100" s="13" t="inlineStr">
         <is>
-          <t>5.2% rostered</t>
+          <t>5.1% rostered</t>
         </is>
       </c>
       <c r="F100" s="17" t="inlineStr">
@@ -8440,12 +8440,12 @@
       </c>
       <c r="D104" s="13" t="inlineStr">
         <is>
-          <t>1.1%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
         <is>
-          <t>1.1% rostered</t>
+          <t>1.0% rostered</t>
         </is>
       </c>
       <c r="F104" s="17" t="inlineStr">
@@ -8746,12 +8746,12 @@
       </c>
       <c r="D108" s="13" t="inlineStr">
         <is>
-          <t>99.8%</t>
+          <t>99.7%</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr">
         <is>
-          <t>99.8% rostered</t>
+          <t>99.7% rostered</t>
         </is>
       </c>
       <c r="F108" s="18" t="inlineStr">
@@ -8900,12 +8900,12 @@
       </c>
       <c r="D110" s="13" t="inlineStr">
         <is>
-          <t>97.7%</t>
+          <t>97.8%</t>
         </is>
       </c>
       <c r="E110" s="13" t="inlineStr">
         <is>
-          <t>97.7% rostered</t>
+          <t>97.8% rostered</t>
         </is>
       </c>
       <c r="F110" s="18" t="inlineStr">
@@ -9054,12 +9054,12 @@
       </c>
       <c r="D112" s="13" t="inlineStr">
         <is>
-          <t>91.2%</t>
+          <t>91.3%</t>
         </is>
       </c>
       <c r="E112" s="13" t="inlineStr">
         <is>
-          <t>91.2% rostered</t>
+          <t>91.3% rostered</t>
         </is>
       </c>
       <c r="F112" s="18" t="inlineStr">
@@ -9131,12 +9131,12 @@
       </c>
       <c r="D113" s="8" t="inlineStr">
         <is>
-          <t>90.7%</t>
+          <t>90.8%</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>90.7% rostered</t>
+          <t>90.8% rostered</t>
         </is>
       </c>
       <c r="F113" s="18" t="inlineStr">
@@ -9206,12 +9206,12 @@
       </c>
       <c r="D114" s="13" t="inlineStr">
         <is>
-          <t>86.6%</t>
+          <t>86.7%</t>
         </is>
       </c>
       <c r="E114" s="13" t="inlineStr">
         <is>
-          <t>86.6% rostered</t>
+          <t>86.7% rostered</t>
         </is>
       </c>
       <c r="F114" s="18" t="inlineStr">
@@ -9283,12 +9283,12 @@
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>85.8%</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>85.7% rostered</t>
+          <t>85.8% rostered</t>
         </is>
       </c>
       <c r="F115" s="18" t="inlineStr">
@@ -9360,12 +9360,12 @@
       </c>
       <c r="D116" s="13" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>84.1%</t>
         </is>
       </c>
       <c r="E116" s="13" t="inlineStr">
         <is>
-          <t>83.8% rostered</t>
+          <t>84.1% rostered</t>
         </is>
       </c>
       <c r="F116" s="18" t="inlineStr">
@@ -9437,12 +9437,12 @@
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>82.4%</t>
+          <t>82.5%</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>82.4% rostered</t>
+          <t>82.5% rostered</t>
         </is>
       </c>
       <c r="F117" s="18" t="inlineStr">
@@ -9514,12 +9514,12 @@
       </c>
       <c r="D118" s="13" t="inlineStr">
         <is>
-          <t>75.5%</t>
+          <t>75.2%</t>
         </is>
       </c>
       <c r="E118" s="13" t="inlineStr">
         <is>
-          <t>75.5% rostered</t>
+          <t>75.2% rostered</t>
         </is>
       </c>
       <c r="F118" s="18" t="inlineStr">
@@ -9576,12 +9576,12 @@
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
@@ -9591,12 +9591,12 @@
       </c>
       <c r="D119" s="8" t="inlineStr">
         <is>
-          <t>74.4%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t>74.4% rostered</t>
+          <t>74.1% rostered</t>
         </is>
       </c>
       <c r="F119" s="18" t="inlineStr">
@@ -9606,22 +9606,22 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>.359</t>
+          <t>.425</t>
         </is>
       </c>
       <c r="H119" s="8" t="inlineStr">
         <is>
-          <t>.356</t>
+          <t>.399</t>
         </is>
       </c>
       <c r="I119" s="11" t="inlineStr">
         <is>
-          <t>-.003</t>
+          <t>-.026</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>.352</t>
+          <t>.316</t>
         </is>
       </c>
       <c r="K119" s="8" t="inlineStr">
@@ -9631,17 +9631,17 @@
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
-          <t>+.055</t>
+          <t>+.019</t>
         </is>
       </c>
       <c r="M119" s="11" t="inlineStr">
         <is>
-          <t>-0.159</t>
+          <t>-0.152</t>
         </is>
       </c>
       <c r="N119" s="8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>35</t>
         </is>
       </c>
       <c r="O119" s="8" t="inlineStr">
@@ -9653,12 +9653,12 @@
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
@@ -9668,12 +9668,12 @@
       </c>
       <c r="D120" s="13" t="inlineStr">
         <is>
-          <t>73.5%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="E120" s="13" t="inlineStr">
         <is>
-          <t>73.5% rostered</t>
+          <t>74.0% rostered</t>
         </is>
       </c>
       <c r="F120" s="18" t="inlineStr">
@@ -9683,22 +9683,22 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>.425</t>
+          <t>.359</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>.399</t>
+          <t>.356</t>
         </is>
       </c>
       <c r="I120" s="15" t="inlineStr">
         <is>
-          <t>-.026</t>
+          <t>-.003</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
         <is>
-          <t>.316</t>
+          <t>.352</t>
         </is>
       </c>
       <c r="K120" s="13" t="inlineStr">
@@ -9708,17 +9708,17 @@
       </c>
       <c r="L120" s="14" t="inlineStr">
         <is>
-          <t>+.019</t>
+          <t>+.055</t>
         </is>
       </c>
       <c r="M120" s="15" t="inlineStr">
         <is>
-          <t>-0.152</t>
+          <t>-0.159</t>
         </is>
       </c>
       <c r="N120" s="13" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>25</t>
         </is>
       </c>
       <c r="O120" s="13" t="inlineStr">
@@ -9745,12 +9745,12 @@
       </c>
       <c r="D121" s="8" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>72.2%</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t>72.4% rostered</t>
+          <t>72.2% rostered</t>
         </is>
       </c>
       <c r="F121" s="18" t="inlineStr">
@@ -9822,12 +9822,12 @@
       </c>
       <c r="D122" s="13" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>61.1%</t>
         </is>
       </c>
       <c r="E122" s="13" t="inlineStr">
         <is>
-          <t>59.0% rostered</t>
+          <t>61.1% rostered</t>
         </is>
       </c>
       <c r="F122" s="18" t="inlineStr">
@@ -9899,12 +9899,12 @@
       </c>
       <c r="D123" s="8" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>39.5%</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
         <is>
-          <t>39.6% rostered</t>
+          <t>39.5% rostered</t>
         </is>
       </c>
       <c r="F123" s="18" t="inlineStr">
@@ -9976,12 +9976,12 @@
       </c>
       <c r="D124" s="13" t="inlineStr">
         <is>
-          <t>38.2%</t>
+          <t>38.6%</t>
         </is>
       </c>
       <c r="E124" s="13" t="inlineStr">
         <is>
-          <t>38.2% rostered</t>
+          <t>38.6% rostered</t>
         </is>
       </c>
       <c r="F124" s="18" t="inlineStr">
@@ -10053,12 +10053,12 @@
       </c>
       <c r="D125" s="8" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
         <is>
-          <t>30.7% rostered</t>
+          <t>30.2% rostered</t>
         </is>
       </c>
       <c r="F125" s="18" t="inlineStr">
@@ -10130,12 +10130,12 @@
       </c>
       <c r="D126" s="13" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="E126" s="13" t="inlineStr">
         <is>
-          <t>26.2% rostered</t>
+          <t>26.1% rostered</t>
         </is>
       </c>
       <c r="F126" s="18" t="inlineStr">
@@ -10284,12 +10284,12 @@
       </c>
       <c r="D128" s="13" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="E128" s="13" t="inlineStr">
         <is>
-          <t>11.8% rostered</t>
+          <t>12.5% rostered</t>
         </is>
       </c>
       <c r="F128" s="18" t="inlineStr">
@@ -10346,12 +10346,12 @@
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B129" s="8" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
@@ -10361,12 +10361,12 @@
       </c>
       <c r="D129" s="8" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
         <is>
-          <t>10.6% rostered</t>
+          <t>11.0% rostered</t>
         </is>
       </c>
       <c r="F129" s="18" t="inlineStr">
@@ -10376,59 +10376,59 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>.389</t>
+          <t>.402</t>
         </is>
       </c>
       <c r="H129" s="8" t="inlineStr">
         <is>
-          <t>.358</t>
+          <t>.399</t>
         </is>
       </c>
       <c r="I129" s="11" t="inlineStr">
         <is>
-          <t>-.031</t>
+          <t>-.003</t>
         </is>
       </c>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>.364</t>
+          <t>.409</t>
         </is>
       </c>
       <c r="K129" s="8" t="inlineStr">
         <is>
-          <t>.280</t>
+          <t>.260</t>
         </is>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
-          <t>+.084</t>
+          <t>+.149</t>
         </is>
       </c>
       <c r="M129" s="11" t="inlineStr">
         <is>
-          <t>-0.214</t>
+          <t>-0.391</t>
         </is>
       </c>
       <c r="N129" s="8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>29</t>
         </is>
       </c>
       <c r="O129" s="8" t="inlineStr">
         <is>
-          <t>Second half fader (amplified)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
@@ -10438,12 +10438,12 @@
       </c>
       <c r="D130" s="13" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="E130" s="13" t="inlineStr">
         <is>
-          <t>10.5% rostered</t>
+          <t>10.4% rostered</t>
         </is>
       </c>
       <c r="F130" s="18" t="inlineStr">
@@ -10453,47 +10453,47 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>.402</t>
+          <t>.389</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr">
         <is>
-          <t>.399</t>
+          <t>.358</t>
         </is>
       </c>
       <c r="I130" s="15" t="inlineStr">
         <is>
-          <t>-.003</t>
+          <t>-.031</t>
         </is>
       </c>
       <c r="J130" s="13" t="inlineStr">
         <is>
-          <t>.409</t>
+          <t>.364</t>
         </is>
       </c>
       <c r="K130" s="13" t="inlineStr">
         <is>
-          <t>.260</t>
+          <t>.280</t>
         </is>
       </c>
       <c r="L130" s="14" t="inlineStr">
         <is>
-          <t>+.149</t>
+          <t>+.084</t>
         </is>
       </c>
       <c r="M130" s="15" t="inlineStr">
         <is>
-          <t>-0.391</t>
+          <t>-0.214</t>
         </is>
       </c>
       <c r="N130" s="13" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>32</t>
         </is>
       </c>
       <c r="O130" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Second half fader (amplified)</t>
         </is>
       </c>
     </row>
@@ -10515,12 +10515,12 @@
       </c>
       <c r="D131" s="8" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>10.1% rostered</t>
+          <t>10.0% rostered</t>
         </is>
       </c>
       <c r="F131" s="18" t="inlineStr">
@@ -10592,12 +10592,12 @@
       </c>
       <c r="D132" s="13" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="E132" s="13" t="inlineStr">
         <is>
-          <t>9.2% rostered</t>
+          <t>9.0% rostered</t>
         </is>
       </c>
       <c r="F132" s="18" t="inlineStr">
@@ -10669,12 +10669,12 @@
       </c>
       <c r="D133" s="8" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>9.0% rostered</t>
+          <t>8.3% rostered</t>
         </is>
       </c>
       <c r="F133" s="18" t="inlineStr">
@@ -10731,12 +10731,12 @@
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Jose Fernandez</t>
         </is>
       </c>
       <c r="B134" s="13" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
@@ -10746,12 +10746,12 @@
       </c>
       <c r="D134" s="13" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="E134" s="13" t="inlineStr">
         <is>
-          <t>7.1% rostered</t>
+          <t>7.2% rostered</t>
         </is>
       </c>
       <c r="F134" s="18" t="inlineStr">
@@ -10761,22 +10761,22 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>.354</t>
+          <t>.394</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr">
         <is>
-          <t>.353</t>
+          <t>.340</t>
         </is>
       </c>
       <c r="I134" s="15" t="inlineStr">
         <is>
-          <t>-.001</t>
+          <t>-.054</t>
         </is>
       </c>
       <c r="J134" s="13" t="inlineStr">
         <is>
-          <t>.432</t>
+          <t>.400</t>
         </is>
       </c>
       <c r="K134" s="13" t="inlineStr">
@@ -10791,12 +10791,12 @@
       </c>
       <c r="M134" s="15" t="inlineStr">
         <is>
-          <t>-0.358</t>
+          <t>-0.212</t>
         </is>
       </c>
       <c r="N134" s="13" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="O134" s="13" t="inlineStr">
@@ -10808,12 +10808,12 @@
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>Jose Fernandez</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
@@ -10823,12 +10823,12 @@
       </c>
       <c r="D135" s="8" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>6.9% rostered</t>
+          <t>7.0% rostered</t>
         </is>
       </c>
       <c r="F135" s="18" t="inlineStr">
@@ -10838,22 +10838,22 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>.394</t>
+          <t>.354</t>
         </is>
       </c>
       <c r="H135" s="8" t="inlineStr">
         <is>
-          <t>.340</t>
+          <t>.353</t>
         </is>
       </c>
       <c r="I135" s="11" t="inlineStr">
         <is>
-          <t>-.054</t>
+          <t>-.001</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>.400</t>
+          <t>.432</t>
         </is>
       </c>
       <c r="K135" s="8" t="inlineStr">
@@ -10868,12 +10868,12 @@
       </c>
       <c r="M135" s="11" t="inlineStr">
         <is>
-          <t>-0.212</t>
+          <t>-0.358</t>
         </is>
       </c>
       <c r="N135" s="8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="O135" s="8" t="inlineStr">
@@ -10900,12 +10900,12 @@
       </c>
       <c r="D136" s="13" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="E136" s="13" t="inlineStr">
         <is>
-          <t>5.8% rostered</t>
+          <t>5.6% rostered</t>
         </is>
       </c>
       <c r="F136" s="18" t="inlineStr">
@@ -10977,12 +10977,12 @@
       </c>
       <c r="D137" s="8" t="inlineStr">
         <is>
-          <t>5.2%</t>
+          <t>5.3%</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
         <is>
-          <t>5.2% rostered</t>
+          <t>5.3% rostered</t>
         </is>
       </c>
       <c r="F137" s="18" t="inlineStr">
@@ -11054,12 +11054,12 @@
       </c>
       <c r="D138" s="13" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.2%</t>
         </is>
       </c>
       <c r="E138" s="13" t="inlineStr">
         <is>
-          <t>5.0% rostered</t>
+          <t>5.2% rostered</t>
         </is>
       </c>
       <c r="F138" s="18" t="inlineStr">
@@ -11131,12 +11131,12 @@
       </c>
       <c r="D139" s="8" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
         <is>
-          <t>4.4% rostered</t>
+          <t>4.2% rostered</t>
         </is>
       </c>
       <c r="F139" s="18" t="inlineStr">
@@ -11208,12 +11208,12 @@
       </c>
       <c r="D140" s="13" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="E140" s="13" t="inlineStr">
         <is>
-          <t>2.1% rostered</t>
+          <t>2.5% rostered</t>
         </is>
       </c>
       <c r="F140" s="18" t="inlineStr">
@@ -11285,12 +11285,12 @@
       </c>
       <c r="D141" s="8" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>1.4%</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
         <is>
-          <t>1.2% rostered</t>
+          <t>1.4% rostered</t>
         </is>
       </c>
       <c r="F141" s="18" t="inlineStr">
@@ -11609,12 +11609,12 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>98.7%</t>
+          <t>98.8%</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>98.7% rostered</t>
+          <t>98.8% rostered</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -11702,12 +11702,12 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>97.3%</t>
+          <t>97.2%</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>97.3% rostered</t>
+          <t>97.2% rostered</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -11795,12 +11795,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>87.8%</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>87.5% rostered</t>
+          <t>87.8% rostered</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -11888,12 +11888,12 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>68.8% rostered</t>
+          <t>68.4% rostered</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -11981,12 +11981,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>26.7% rostered</t>
+          <t>26.5% rostered</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -12074,12 +12074,12 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>5.3%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>5.3% rostered</t>
+          <t>5.1% rostered</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -12353,12 +12353,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>96.2%</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>96.0% rostered</t>
+          <t>96.2% rostered</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -12446,12 +12446,12 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>55.4%</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>56.0% rostered</t>
+          <t>55.4% rostered</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
@@ -12539,12 +12539,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>24.2%</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>24.8% rostered</t>
+          <t>24.2% rostered</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
@@ -12632,12 +12632,12 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>21.0% rostered</t>
+          <t>21.8% rostered</t>
         </is>
       </c>
       <c r="F16" s="16" t="inlineStr">
@@ -12725,12 +12725,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>2.7% rostered</t>
+          <t>2.6% rostered</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -12911,12 +12911,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>95.5%</t>
+          <t>95.6%</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>95.5% rostered</t>
+          <t>95.6% rostered</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -12989,17 +12989,17 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Chase Burns</t>
+          <t>Gavin Williams</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>33.7</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -13019,47 +13019,47 @@
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>3.34</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>3.72</t>
+          <t>4.38</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>2.73</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="J20" s="15" t="inlineStr">
         <is>
-          <t>-1.05</t>
+          <t>-1.04</t>
         </is>
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>.259</t>
+          <t>.192</t>
         </is>
       </c>
       <c r="L20" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.270</t>
         </is>
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>88.5%</t>
+          <t>81.3%</t>
         </is>
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>-0.083</t>
+          <t>-0.101</t>
         </is>
       </c>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>27</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
@@ -13082,27 +13082,27 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Gavin Williams</t>
+          <t>Chase Burns</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>33.7</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>90.6%</t>
+          <t>90.8%</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>90.6% rostered</t>
+          <t>90.8% rostered</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -13112,47 +13112,47 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>3.34</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>4.38</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-1.05</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>.192</t>
+          <t>.259</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>.270</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
         <is>
-          <t>81.3%</t>
+          <t>88.5%</t>
         </is>
       </c>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>-0.101</t>
+          <t>-0.083</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>23</t>
         </is>
       </c>
       <c r="P21" s="8" t="inlineStr">
@@ -13190,12 +13190,12 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>71.2%</t>
+          <t>71.7%</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>71.2% rostered</t>
+          <t>71.7% rostered</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr">
@@ -13283,12 +13283,12 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>69.0%</t>
+          <t>70.5%</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>69.0% rostered</t>
+          <t>70.5% rostered</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -13376,12 +13376,12 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>55.1%</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>56.0% rostered</t>
+          <t>55.1% rostered</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
@@ -13469,12 +13469,12 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>12.3% rostered</t>
+          <t>12.2% rostered</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
@@ -13562,12 +13562,12 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>6.8% rostered</t>
+          <t>7.0% rostered</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
@@ -13655,12 +13655,12 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>1.1%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>1.1% rostered</t>
+          <t>1.0% rostered</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -13748,12 +13748,12 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>99.9%</t>
+          <t>99.8%</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>99.9% rostered</t>
+          <t>99.8% rostered</t>
         </is>
       </c>
       <c r="F28" s="18" t="inlineStr">
@@ -14027,12 +14027,12 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>85.2%</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>84.9% rostered</t>
+          <t>85.2% rostered</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -14120,12 +14120,12 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>77.3%</t>
+          <t>77.4%</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>77.3% rostered</t>
+          <t>77.4% rostered</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
@@ -14213,12 +14213,12 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>70.5%</t>
+          <t>72.3%</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>70.5% rostered</t>
+          <t>72.3% rostered</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
@@ -14306,12 +14306,12 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>69.3%</t>
+          <t>68.9%</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>69.3% rostered</t>
+          <t>68.9% rostered</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
@@ -14399,12 +14399,12 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>52.8% rostered</t>
+          <t>51.5% rostered</t>
         </is>
       </c>
       <c r="F35" s="18" t="inlineStr">
@@ -14492,12 +14492,12 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>45.4%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>45.4% rostered</t>
+          <t>46.0% rostered</t>
         </is>
       </c>
       <c r="F36" s="18" t="inlineStr">
@@ -14585,12 +14585,12 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>44.3%</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>43.8% rostered</t>
+          <t>44.3% rostered</t>
         </is>
       </c>
       <c r="F37" s="18" t="inlineStr">
@@ -14678,12 +14678,12 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>35.7%</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>35.3% rostered</t>
+          <t>35.7% rostered</t>
         </is>
       </c>
       <c r="F38" s="18" t="inlineStr">
@@ -14771,12 +14771,12 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>24.5% rostered</t>
+          <t>26.1% rostered</t>
         </is>
       </c>
       <c r="F39" s="18" t="inlineStr">
@@ -14864,12 +14864,12 @@
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>24.0% rostered</t>
+          <t>23.9% rostered</t>
         </is>
       </c>
       <c r="F40" s="18" t="inlineStr">
@@ -14957,12 +14957,12 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>21.0% rostered</t>
+          <t>21.8% rostered</t>
         </is>
       </c>
       <c r="F41" s="18" t="inlineStr">
@@ -15050,12 +15050,12 @@
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>18.6% rostered</t>
+          <t>18.9% rostered</t>
         </is>
       </c>
       <c r="F42" s="18" t="inlineStr">
@@ -15128,27 +15128,27 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Nick Martínez</t>
+          <t>Eduardo Rodríguez</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>TB</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>17.7% rostered</t>
+          <t>18.7% rostered</t>
         </is>
       </c>
       <c r="F43" s="18" t="inlineStr">
@@ -15158,47 +15158,47 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>4.90</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>3.68</t>
+          <t>4.97</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>-2.06</t>
+          <t>-2.01</t>
         </is>
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>.227</t>
+          <t>.244</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>.292</t>
+          <t>.306</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>94.0%</t>
+          <t>87.6%</t>
         </is>
       </c>
       <c r="N43" s="11" t="inlineStr">
         <is>
-          <t>-0.469</t>
+          <t>-0.251</t>
         </is>
       </c>
       <c r="O43" s="8" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>33</t>
         </is>
       </c>
       <c r="P43" s="8" t="inlineStr">
@@ -15221,27 +15221,27 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>Eduardo Rodríguez</t>
+          <t>Nick Martínez</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>17.1% rostered</t>
+          <t>18.2% rostered</t>
         </is>
       </c>
       <c r="F44" s="18" t="inlineStr">
@@ -15251,47 +15251,47 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>4.90</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>4.97</t>
+          <t>3.68</t>
         </is>
       </c>
       <c r="J44" s="15" t="inlineStr">
         <is>
-          <t>-2.01</t>
+          <t>-2.06</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>.244</t>
+          <t>.227</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>.306</t>
+          <t>.292</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr">
         <is>
-          <t>87.6%</t>
+          <t>94.0%</t>
         </is>
       </c>
       <c r="N44" s="15" t="inlineStr">
         <is>
-          <t>-0.251</t>
+          <t>-0.469</t>
         </is>
       </c>
       <c r="O44" s="13" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>36</t>
         </is>
       </c>
       <c r="P44" s="13" t="inlineStr">
@@ -15329,12 +15329,12 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>12.9% rostered</t>
+          <t>11.9% rostered</t>
         </is>
       </c>
       <c r="F45" s="18" t="inlineStr">
@@ -15422,12 +15422,12 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>8.2% rostered</t>
+          <t>8.0% rostered</t>
         </is>
       </c>
       <c r="F46" s="18" t="inlineStr">
@@ -15515,12 +15515,12 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>7.9% rostered</t>
+          <t>7.8% rostered</t>
         </is>
       </c>
       <c r="F47" s="18" t="inlineStr">
@@ -15593,27 +15593,27 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>Aaron Civale</t>
+          <t>Tomoyuki Sugano</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>30.3</t>
+          <t>26.3</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>5.4% rostered</t>
+          <t>6.0% rostered</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
@@ -15623,52 +15623,52 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>3.42</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>4.62</t>
+          <t>6.08</t>
         </is>
       </c>
       <c r="J48" s="15" t="inlineStr">
         <is>
-          <t>-0.86</t>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>.305</t>
+          <t>.241</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
         <is>
-          <t>.294</t>
+          <t>.324</t>
         </is>
       </c>
       <c r="M48" s="13" t="inlineStr">
         <is>
-          <t>85.4%</t>
+          <t>83.3%</t>
         </is>
       </c>
       <c r="N48" s="15" t="inlineStr">
         <is>
-          <t>-0.156</t>
+          <t>-0.242</t>
         </is>
       </c>
       <c r="O48" s="13" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>37</t>
         </is>
       </c>
       <c r="P48" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q48" s="13" t="inlineStr">
@@ -15686,27 +15686,27 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Tomoyuki Sugano</t>
+          <t>Aaron Civale</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>26.3</t>
+          <t>30.3</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>5.2%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>5.2% rostered</t>
+          <t>5.1% rostered</t>
         </is>
       </c>
       <c r="F49" s="18" t="inlineStr">
@@ -15716,52 +15716,52 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>6.08</t>
+          <t>4.62</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t>-0.86</t>
         </is>
       </c>
       <c r="K49" s="8" t="inlineStr">
         <is>
-          <t>.241</t>
+          <t>.305</t>
         </is>
       </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>.324</t>
+          <t>.294</t>
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>85.4%</t>
         </is>
       </c>
       <c r="N49" s="11" t="inlineStr">
         <is>
-          <t>-0.242</t>
+          <t>-0.156</t>
         </is>
       </c>
       <c r="O49" s="8" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>31</t>
         </is>
       </c>
       <c r="P49" s="8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q49" s="8" t="inlineStr">
@@ -15794,12 +15794,12 @@
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>3.6% rostered</t>
+          <t>3.3% rostered</t>
         </is>
       </c>
       <c r="F50" s="18" t="inlineStr">
@@ -16284,12 +16284,12 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>99.8%</t>
+          <t>99.7%</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>99.8% rostered</t>
+          <t>99.7% rostered</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
@@ -16408,12 +16408,12 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>99.4%</t>
+          <t>99.5%</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>99.4% rostered</t>
+          <t>99.5% rostered</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
@@ -16656,12 +16656,12 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>97.7%</t>
+          <t>97.8%</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>97.7% rostered</t>
+          <t>97.8% rostered</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -16780,12 +16780,12 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>97.2%</t>
+          <t>97.3%</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>97.2% rostered</t>
+          <t>97.3% rostered</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
@@ -17090,12 +17090,12 @@
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>94.4%</t>
+          <t>94.5%</t>
         </is>
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>94.4% rostered</t>
+          <t>94.5% rostered</t>
         </is>
       </c>
       <c r="F21" s="24" t="inlineStr">
@@ -17214,12 +17214,12 @@
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>92.8%</t>
+          <t>93.0%</t>
         </is>
       </c>
       <c r="E23" s="24" t="inlineStr">
         <is>
-          <t>92.8% rostered</t>
+          <t>93.0% rostered</t>
         </is>
       </c>
       <c r="F23" s="24" t="inlineStr">
@@ -17276,12 +17276,12 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>92.2%</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>92.3% rostered</t>
+          <t>92.2% rostered</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
@@ -17338,12 +17338,12 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>90.7%</t>
+          <t>90.8%</t>
         </is>
       </c>
       <c r="E25" s="24" t="inlineStr">
         <is>
-          <t>90.7% rostered</t>
+          <t>90.8% rostered</t>
         </is>
       </c>
       <c r="F25" s="24" t="inlineStr">
@@ -17400,12 +17400,12 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>88.5%</t>
+          <t>88.6%</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>88.5% rostered</t>
+          <t>88.6% rostered</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr">
@@ -17447,7 +17447,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="23" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
@@ -17462,54 +17462,54 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>86.6%</t>
+          <t>86.9%</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>86.6% rostered</t>
+          <t>86.9% rostered</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>.386</t>
+          <t>.396</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>.417</t>
+          <t>.413</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
         <is>
-          <t>.394</t>
+          <t>.345</t>
         </is>
       </c>
       <c r="I27" s="24" t="inlineStr">
         <is>
-          <t>.314</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J27" s="28" t="inlineStr">
         <is>
-          <t>-0.223</t>
-        </is>
-      </c>
-      <c r="K27" s="18" t="inlineStr">
-        <is>
-          <t>Sell high</t>
+          <t>-0.072</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L27" s="24" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
@@ -17524,47 +17524,47 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>86.5%</t>
+          <t>86.7%</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>86.5% rostered</t>
+          <t>86.7% rostered</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>.396</t>
+          <t>.386</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>.413</t>
+          <t>.417</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>.345</t>
+          <t>.394</t>
         </is>
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>.314</t>
         </is>
       </c>
       <c r="J28" s="15" t="inlineStr">
         <is>
-          <t>-0.072</t>
-        </is>
-      </c>
-      <c r="K28" s="7" t="inlineStr">
-        <is>
-          <t>Neutral</t>
+          <t>-0.223</t>
+        </is>
+      </c>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>Sell high</t>
         </is>
       </c>
       <c r="L28" s="13" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
     </row>
@@ -17586,12 +17586,12 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>85.9%</t>
+          <t>86.0%</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>85.9% rostered</t>
+          <t>86.0% rostered</t>
         </is>
       </c>
       <c r="F29" s="24" t="inlineStr">
@@ -17648,12 +17648,12 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>85.8%</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>85.7% rostered</t>
+          <t>85.8% rostered</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
@@ -17695,32 +17695,32 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="C31" s="25" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>84.0%</t>
+          <t>84.1%</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>84.0% rostered</t>
+          <t>84.1% rostered</t>
         </is>
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>.378</t>
+          <t>.427</t>
         </is>
       </c>
       <c r="G31" s="24" t="inlineStr">
@@ -17730,106 +17730,106 @@
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
-          <t>.278</t>
+          <t>.395</t>
         </is>
       </c>
       <c r="I31" s="24" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J31" s="26" t="inlineStr">
-        <is>
-          <t>+0.049</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr">
-        <is>
-          <t>Neutral</t>
+          <t>.319</t>
+        </is>
+      </c>
+      <c r="J31" s="28" t="inlineStr">
+        <is>
+          <t>-0.151</t>
+        </is>
+      </c>
+      <c r="K31" s="18" t="inlineStr">
+        <is>
+          <t>Sell high</t>
         </is>
       </c>
       <c r="L31" s="24" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>CHC</t>
-        </is>
-      </c>
-      <c r="C32" s="27" t="inlineStr">
-        <is>
-          <t>Monitor</t>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>83.7%</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>83.8% rostered</t>
+          <t>83.7% rostered</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
+          <t>.378</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
           <t>.427</t>
         </is>
       </c>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>.427</t>
-        </is>
-      </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>.395</t>
+          <t>.278</t>
         </is>
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>.319</t>
-        </is>
-      </c>
-      <c r="J32" s="15" t="inlineStr">
-        <is>
-          <t>-0.151</t>
-        </is>
-      </c>
-      <c r="K32" s="18" t="inlineStr">
-        <is>
-          <t>Sell high</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J32" s="14" t="inlineStr">
+        <is>
+          <t>+0.049</t>
+        </is>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L32" s="13" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>CHC</t>
-        </is>
-      </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D33" s="24" t="inlineStr">
@@ -17844,54 +17844,54 @@
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>.373</t>
+          <t>.404</t>
         </is>
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
-          <t>.350</t>
+          <t>.395</t>
         </is>
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>.270</t>
+          <t>.368</t>
         </is>
       </c>
       <c r="I33" s="24" t="inlineStr">
         <is>
-          <t>.301</t>
+          <t>.291</t>
         </is>
       </c>
       <c r="J33" s="28" t="inlineStr">
         <is>
-          <t>-0.011</t>
-        </is>
-      </c>
-      <c r="K33" s="7" t="inlineStr">
-        <is>
-          <t>Neutral</t>
+          <t>-0.265</t>
+        </is>
+      </c>
+      <c r="K33" s="18" t="inlineStr">
+        <is>
+          <t>Sell high</t>
         </is>
       </c>
       <c r="L33" s="24" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="C34" s="27" t="inlineStr">
-        <is>
-          <t>Monitor</t>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="C34" s="25" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -17906,37 +17906,37 @@
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>.404</t>
+          <t>.373</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>.395</t>
+          <t>.350</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>.368</t>
+          <t>.270</t>
         </is>
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>.291</t>
+          <t>.301</t>
         </is>
       </c>
       <c r="J34" s="15" t="inlineStr">
         <is>
-          <t>-0.265</t>
-        </is>
-      </c>
-      <c r="K34" s="18" t="inlineStr">
-        <is>
-          <t>Sell high</t>
+          <t>-0.011</t>
+        </is>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L34" s="13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>32</t>
         </is>
       </c>
     </row>
@@ -17958,12 +17958,12 @@
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>81.4%</t>
+          <t>81.7%</t>
         </is>
       </c>
       <c r="E35" s="24" t="inlineStr">
         <is>
-          <t>81.4% rostered</t>
+          <t>81.7% rostered</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
@@ -18020,12 +18020,12 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>78.5%</t>
+          <t>78.9%</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>78.5% rostered</t>
+          <t>78.9% rostered</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
@@ -18082,12 +18082,12 @@
       </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
-          <t>73.5%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="E37" s="24" t="inlineStr">
         <is>
-          <t>73.5% rostered</t>
+          <t>74.1% rostered</t>
         </is>
       </c>
       <c r="F37" s="24" t="inlineStr">
@@ -18144,12 +18144,12 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>72.2%</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>72.4% rostered</t>
+          <t>72.2% rostered</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
@@ -18206,12 +18206,12 @@
       </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>63.3%</t>
         </is>
       </c>
       <c r="E39" s="24" t="inlineStr">
         <is>
-          <t>63.4% rostered</t>
+          <t>63.3% rostered</t>
         </is>
       </c>
       <c r="F39" s="24" t="inlineStr">
@@ -18268,12 +18268,12 @@
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>61.1%</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>59.0% rostered</t>
+          <t>61.1% rostered</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr">
@@ -18330,12 +18330,12 @@
       </c>
       <c r="D41" s="24" t="inlineStr">
         <is>
-          <t>57.7%</t>
+          <t>57.9%</t>
         </is>
       </c>
       <c r="E41" s="24" t="inlineStr">
         <is>
-          <t>57.7% rostered</t>
+          <t>57.9% rostered</t>
         </is>
       </c>
       <c r="F41" s="24" t="inlineStr">
@@ -18392,12 +18392,12 @@
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>40.5%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>40.5% rostered</t>
+          <t>40.6% rostered</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr">
@@ -18454,12 +18454,12 @@
       </c>
       <c r="D43" s="24" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>31.1%</t>
         </is>
       </c>
       <c r="E43" s="24" t="inlineStr">
         <is>
-          <t>30.1% rostered</t>
+          <t>31.1% rostered</t>
         </is>
       </c>
       <c r="F43" s="24" t="inlineStr">
@@ -18516,12 +18516,12 @@
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>28.0% rostered</t>
+          <t>29.4% rostered</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
@@ -18563,12 +18563,12 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Iván Herrera</t>
         </is>
       </c>
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="C45" s="25" t="inlineStr">
@@ -18578,171 +18578,171 @@
       </c>
       <c r="D45" s="24" t="inlineStr">
         <is>
-          <t>26.1%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>26.1% rostered</t>
+          <t>26.7% rostered</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>.383</t>
+          <t>.380</t>
         </is>
       </c>
       <c r="G45" s="24" t="inlineStr">
         <is>
-          <t>.372</t>
+          <t>.423</t>
         </is>
       </c>
       <c r="H45" s="24" t="inlineStr">
         <is>
-          <t>.308</t>
+          <t>.270</t>
         </is>
       </c>
       <c r="I45" s="24" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J45" s="28" t="inlineStr">
-        <is>
-          <t>-0.040</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr">
-        <is>
-          <t>Neutral</t>
+          <t>.340</t>
+        </is>
+      </c>
+      <c r="J45" s="26" t="inlineStr">
+        <is>
+          <t>+0.365</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>Buy low</t>
         </is>
       </c>
       <c r="L45" s="24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>Willson Contreras</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>BOS</t>
-        </is>
-      </c>
-      <c r="C46" s="27" t="inlineStr">
-        <is>
-          <t>Monitor</t>
+          <t>KC</t>
+        </is>
+      </c>
+      <c r="C46" s="25" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>25.7% rostered</t>
+          <t>26.1% rostered</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>.373</t>
+          <t>.383</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>.402</t>
+          <t>.372</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>.339</t>
+          <t>.308</t>
         </is>
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>.306</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J46" s="15" t="inlineStr">
         <is>
-          <t>-0.141</t>
-        </is>
-      </c>
-      <c r="K46" s="17" t="inlineStr">
-        <is>
-          <t>Slight sell</t>
+          <t>-0.040</t>
+        </is>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L46" s="13" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>Iván Herrera</t>
+          <t>Willson Contreras</t>
         </is>
       </c>
       <c r="B47" s="24" t="inlineStr">
         <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="C47" s="25" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="C47" s="27" t="inlineStr">
+        <is>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="E47" s="24" t="inlineStr">
         <is>
-          <t>25.0% rostered</t>
+          <t>25.8% rostered</t>
         </is>
       </c>
       <c r="F47" s="24" t="inlineStr">
         <is>
-          <t>.380</t>
+          <t>.373</t>
         </is>
       </c>
       <c r="G47" s="24" t="inlineStr">
         <is>
-          <t>.423</t>
+          <t>.402</t>
         </is>
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
-          <t>.270</t>
+          <t>.339</t>
         </is>
       </c>
       <c r="I47" s="24" t="inlineStr">
         <is>
-          <t>.340</t>
-        </is>
-      </c>
-      <c r="J47" s="26" t="inlineStr">
-        <is>
-          <t>+0.365</t>
-        </is>
-      </c>
-      <c r="K47" s="9" t="inlineStr">
-        <is>
-          <t>Buy low</t>
+          <t>.306</t>
+        </is>
+      </c>
+      <c r="J47" s="28" t="inlineStr">
+        <is>
+          <t>-0.141</t>
+        </is>
+      </c>
+      <c r="K47" s="17" t="inlineStr">
+        <is>
+          <t>Slight sell</t>
         </is>
       </c>
       <c r="L47" s="24" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>34</t>
         </is>
       </c>
     </row>
@@ -18764,12 +18764,12 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>20.7% rostered</t>
+          <t>22.8% rostered</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
@@ -18826,12 +18826,12 @@
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>17.1% rostered</t>
+          <t>17.7% rostered</t>
         </is>
       </c>
       <c r="F49" s="24" t="inlineStr">
@@ -18950,12 +18950,12 @@
       </c>
       <c r="D51" s="24" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="E51" s="24" t="inlineStr">
         <is>
-          <t>11.8% rostered</t>
+          <t>12.5% rostered</t>
         </is>
       </c>
       <c r="F51" s="24" t="inlineStr">
@@ -18997,12 +18997,12 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C52" s="27" t="inlineStr">
@@ -19012,37 +19012,37 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>10.6% rostered</t>
+          <t>11.0% rostered</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>.389</t>
+          <t>.402</t>
         </is>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>.358</t>
+          <t>.399</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>.364</t>
+          <t>.409</t>
         </is>
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>.280</t>
+          <t>.260</t>
         </is>
       </c>
       <c r="J52" s="15" t="inlineStr">
         <is>
-          <t>-0.214</t>
+          <t>-0.391</t>
         </is>
       </c>
       <c r="K52" s="18" t="inlineStr">
@@ -19052,19 +19052,19 @@
       </c>
       <c r="L52" s="13" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="23" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B53" s="24" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="C53" s="27" t="inlineStr">
@@ -19074,37 +19074,37 @@
       </c>
       <c r="D53" s="24" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="E53" s="24" t="inlineStr">
         <is>
-          <t>10.5% rostered</t>
+          <t>10.4% rostered</t>
         </is>
       </c>
       <c r="F53" s="24" t="inlineStr">
         <is>
-          <t>.402</t>
+          <t>.389</t>
         </is>
       </c>
       <c r="G53" s="24" t="inlineStr">
         <is>
-          <t>.399</t>
+          <t>.358</t>
         </is>
       </c>
       <c r="H53" s="24" t="inlineStr">
         <is>
-          <t>.409</t>
+          <t>.364</t>
         </is>
       </c>
       <c r="I53" s="24" t="inlineStr">
         <is>
-          <t>.260</t>
+          <t>.280</t>
         </is>
       </c>
       <c r="J53" s="28" t="inlineStr">
         <is>
-          <t>-0.391</t>
+          <t>-0.214</t>
         </is>
       </c>
       <c r="K53" s="18" t="inlineStr">
@@ -19114,7 +19114,7 @@
       </c>
       <c r="L53" s="24" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>32</t>
         </is>
       </c>
     </row>
@@ -19136,12 +19136,12 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>9.0% rostered</t>
+          <t>8.3% rostered</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
@@ -19198,12 +19198,12 @@
       </c>
       <c r="D55" s="24" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="E55" s="24" t="inlineStr">
         <is>
-          <t>8.2% rostered</t>
+          <t>8.0% rostered</t>
         </is>
       </c>
       <c r="F55" s="24" t="inlineStr">
@@ -19260,12 +19260,12 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>6.9% rostered</t>
+          <t>7.2% rostered</t>
         </is>
       </c>
       <c r="F56" s="13" t="inlineStr">
@@ -19322,12 +19322,12 @@
       </c>
       <c r="D57" s="24" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="E57" s="24" t="inlineStr">
         <is>
-          <t>6.6% rostered</t>
+          <t>6.5% rostered</t>
         </is>
       </c>
       <c r="F57" s="24" t="inlineStr">
@@ -19384,12 +19384,12 @@
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.2%</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
         <is>
-          <t>5.0% rostered</t>
+          <t>5.2% rostered</t>
         </is>
       </c>
       <c r="F58" s="13" t="inlineStr">
@@ -19493,12 +19493,12 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>Miguel Andújar</t>
+          <t>Edouard Julien</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="C60" s="27" t="inlineStr">
@@ -19508,59 +19508,59 @@
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>1.4%</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>1.2% rostered</t>
+          <t>1.4% rostered</t>
         </is>
       </c>
       <c r="F60" s="13" t="inlineStr">
         <is>
-          <t>.372</t>
+          <t>.374</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>.283</t>
+          <t>.388</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t>.417</t>
+          <t>.407</t>
         </is>
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>.337</t>
+          <t>.281</t>
         </is>
       </c>
       <c r="J60" s="15" t="inlineStr">
         <is>
-          <t>-0.132</t>
-        </is>
-      </c>
-      <c r="K60" s="17" t="inlineStr">
-        <is>
-          <t>Slight sell</t>
+          <t>-0.209</t>
+        </is>
+      </c>
+      <c r="K60" s="18" t="inlineStr">
+        <is>
+          <t>Sell high</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="23" t="inlineStr">
         <is>
-          <t>Edouard Julien</t>
+          <t>Miguel Andújar</t>
         </is>
       </c>
       <c r="B61" s="24" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="C61" s="27" t="inlineStr">
@@ -19580,37 +19580,37 @@
       </c>
       <c r="F61" s="24" t="inlineStr">
         <is>
-          <t>.374</t>
+          <t>.372</t>
         </is>
       </c>
       <c r="G61" s="24" t="inlineStr">
         <is>
-          <t>.388</t>
+          <t>.283</t>
         </is>
       </c>
       <c r="H61" s="24" t="inlineStr">
         <is>
-          <t>.407</t>
+          <t>.417</t>
         </is>
       </c>
       <c r="I61" s="24" t="inlineStr">
         <is>
-          <t>.281</t>
+          <t>.337</t>
         </is>
       </c>
       <c r="J61" s="28" t="inlineStr">
         <is>
-          <t>-0.209</t>
-        </is>
-      </c>
-      <c r="K61" s="18" t="inlineStr">
-        <is>
-          <t>Sell high</t>
+          <t>-0.132</t>
+        </is>
+      </c>
+      <c r="K61" s="17" t="inlineStr">
+        <is>
+          <t>Slight sell</t>
         </is>
       </c>
       <c r="L61" s="24" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -19632,12 +19632,12 @@
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>1.1%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>1.1% rostered</t>
+          <t>1.0% rostered</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
@@ -19821,12 +19821,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>88.8%</t>
+          <t>88.9%</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>88.8% rostered</t>
+          <t>88.9% rostered</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -19888,12 +19888,12 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>73.6%</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>74.0% rostered</t>
+          <t>73.6% rostered</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
@@ -19955,12 +19955,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>61.4%</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>61.8% rostered</t>
+          <t>61.4% rostered</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -20089,12 +20089,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>4.0% rostered</t>
+          <t>3.9% rostered</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -20223,12 +20223,12 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>2.0% rostered</t>
+          <t>1.9% rostered</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -20290,12 +20290,12 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>1.4%</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>1.5% rostered</t>
+          <t>1.4% rostered</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
@@ -20692,12 +20692,12 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>66.0%</t>
+          <t>65.9%</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>66.0% rostered</t>
+          <t>65.9% rostered</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
@@ -20759,12 +20759,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>45.1%</t>
+          <t>45.2%</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>45.1% rostered</t>
+          <t>45.2% rostered</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">

</xml_diff>